<commit_message>
Removed gridlines for dashboard
</commit_message>
<xml_diff>
--- a/excelrestaurent.xlsx
+++ b/excelrestaurent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anjal\OneDrive_backup\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ajayExcel\EuropeanRestaurantDealers\ExcelforDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7151070-FD6E-44B1-94E0-56137C45CE05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2B4066-A9B0-41E7-8650-3C72977E5969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="177" firstSheet="4" activeTab="4" xr2:uid="{2649B7B7-2BEC-4695-85BD-2C8E686F05BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="177" xr2:uid="{2649B7B7-2BEC-4695-85BD-2C8E686F05BA}"/>
   </bookViews>
   <sheets>
     <sheet name="pivot dashboard" sheetId="8" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1348" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1354" uniqueCount="62">
   <si>
     <t>Order ID</t>
   </si>
@@ -1309,7 +1309,7 @@
                 <c:formatCode>#,##0.00_-\ [$€-1]</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>7400.0132999999996</c:v>
+                  <c:v>376999.80689999979</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1876,23 +1876,329 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet4!$A$4:$A$5</c:f>
+              <c:f>Sheet4!$A$4:$A$56</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="52"/>
                 <c:pt idx="0">
-                  <c:v>08-11-2022</c:v>
+                  <c:v>11/8/2022</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11/9/2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11/10/2022</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11/11/2022</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11/12/2022</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>11/13/2022</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>11/14/2022</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>11/15/2022</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>11/16/2022</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11/17/2022</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11/18/2022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11/19/2022</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>11/20/2022</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>11/21/2022</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>11/22/2022</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>11/23/2022</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>11/24/2022</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>11/25/2022</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>11/26/2022</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>11/27/2022</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>11/28/2022</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>11/29/2022</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>11/30/2022</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>12/1/2022</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>12/2/2022</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>12/3/2022</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>12/4/2022</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>12/5/2022</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>12/6/2022</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12/7/2022</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>12/8/2022</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>12/9/2022</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>12/10/2022</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>12/11/2022</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>12/12/2022</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>12/13/2022</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>12/14/2022</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>12/15/2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>12/16/2022</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>12/17/2022</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>12/18/2022</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>12/19/2022</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>12/20/2022</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>12/21/2022</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>12/22/2022</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>12/23/2022</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>12/24/2022</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>12/25/2022</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>12/26/2022</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>12/27/2022</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>12/28/2022</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>12/29/2022</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet4!$B$4:$B$5</c:f>
+              <c:f>Sheet4!$B$4:$B$56</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="52"/>
                 <c:pt idx="0">
                   <c:v>569.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>554.27</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>554.27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>554.27</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>523.48</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>508.08</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>523.48</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>508.08</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>508.08</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>523.48</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>538.88</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>508.08</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>477.29</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>492.69</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>461.89</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>477.29</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>477.29</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>461.89</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>446.5</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>461.89</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>477.29</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>477.29</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>492.69</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>492.69</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>523.48</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>523.48</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>538.88</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>554.27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>538.88</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>523.48</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>538.88</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>569.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>569.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>585.07000000000005</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>569.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>569.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>554.27</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>538.88</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>569.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>585.07000000000005</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>600.46</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>631.25</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>646.65</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>677.44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>677.44</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>646.65</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>677.44</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>677.44</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>692.84</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>692.84</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>723.63</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>754.43</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1929,22 +2235,328 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet4!$A$4:$A$5</c:f>
+              <c:f>Sheet4!$A$4:$A$56</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="52"/>
                 <c:pt idx="0">
-                  <c:v>08-11-2022</c:v>
+                  <c:v>11/8/2022</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11/9/2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11/10/2022</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11/11/2022</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11/12/2022</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>11/13/2022</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>11/14/2022</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>11/15/2022</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>11/16/2022</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11/17/2022</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11/18/2022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11/19/2022</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>11/20/2022</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>11/21/2022</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>11/22/2022</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>11/23/2022</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>11/24/2022</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>11/25/2022</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>11/26/2022</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>11/27/2022</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>11/28/2022</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>11/29/2022</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>11/30/2022</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>12/1/2022</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>12/2/2022</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>12/3/2022</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>12/4/2022</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>12/5/2022</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>12/6/2022</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12/7/2022</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>12/8/2022</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>12/9/2022</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>12/10/2022</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>12/11/2022</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>12/12/2022</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>12/13/2022</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>12/14/2022</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>12/15/2022</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>12/16/2022</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>12/17/2022</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>12/18/2022</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>12/19/2022</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>12/20/2022</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>12/21/2022</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>12/22/2022</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>12/23/2022</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>12/24/2022</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>12/25/2022</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>12/26/2022</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>12/27/2022</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>12/28/2022</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>12/29/2022</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet4!$C$4:$C$5</c:f>
+              <c:f>Sheet4!$C$4:$C$56</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="52"/>
                 <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="51">
                   <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
@@ -2396,23 +3008,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet10!$A$4:$A$5</c:f>
+              <c:f>Sheet10!$A$4:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>Berlin</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Lisbon</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>London</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Madrid</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Paris</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet10!$B$4:$B$5</c:f>
+              <c:f>Sheet10!$B$4:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00_-\ [$€-1]</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>7400.0132999999996</c:v>
+                  <c:v>53399.941500000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>108799.82340000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>101800.29180000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>73599.781199999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>39399.968999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2929,7 +3565,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent4"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln w="19050">
                 <a:solidFill>
@@ -2947,6 +3583,17 @@
           <c:dPt>
             <c:idx val="1"/>
             <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-151B-44AE-B318-F3DDDDFB5019}"/>
@@ -2956,6 +3603,17 @@
           <c:dPt>
             <c:idx val="2"/>
             <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000005-151B-44AE-B318-F3DDDDFB5019}"/>
@@ -2964,23 +3622,35 @@
           </c:dPt>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet2!$A$4:$A$5</c:f>
+              <c:f>Sheet2!$A$4:$A$7</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v> Cash</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v> Credit Card</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v> Gift Card</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$B$4:$B$5</c:f>
+              <c:f>Sheet2!$B$4:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10499,7 +11169,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD8F9540-1C4E-4570-BDF3-9537010ACA75}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="25" rowHeaderCaption="Payment Method Distribution">
-  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
@@ -10527,9 +11197,9 @@
     </pivotField>
     <pivotField axis="axisRow" showAll="0">
       <items count="4">
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10537,10 +11207,10 @@
     <pivotField showAll="0">
       <items count="6">
         <item x="1"/>
-        <item h="1" x="0"/>
-        <item h="1" x="2"/>
-        <item h="1" x="4"/>
-        <item h="1" x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10548,9 +11218,15 @@
   <rowFields count="1">
     <field x="8"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
     </i>
     <i t="grand">
       <x/>
@@ -10712,9 +11388,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10722,10 +11398,10 @@
     <pivotField showAll="0">
       <items count="6">
         <item x="1"/>
-        <item h="1" x="0"/>
-        <item h="1" x="2"/>
-        <item h="1" x="4"/>
-        <item h="1" x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10775,7 +11451,7 @@
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{229F1377-EC9E-484B-8B96-AB5BD0714EE6}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="City">
-  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -10796,9 +11472,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10819,10 +11495,10 @@
     <pivotField axis="axisRow" showAll="0">
       <items count="6">
         <item x="1"/>
-        <item h="1" x="0"/>
-        <item h="1" x="2"/>
-        <item h="1" x="4"/>
-        <item h="1" x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10830,9 +11506,21 @@
   <rowFields count="1">
     <field x="10"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="6">
     <i>
       <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
     </i>
     <i t="grand">
       <x/>
@@ -10872,7 +11560,7 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{598EB335-908B-4C60-A411-3D1E55B023CD}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="20" rowHeaderCaption="Date of purchase">
-  <location ref="A3:C5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <location ref="A3:C56" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -10950,9 +11638,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10973,10 +11661,10 @@
     <pivotField showAll="0">
       <items count="6">
         <item x="1"/>
-        <item h="1" x="0"/>
-        <item h="1" x="2"/>
-        <item h="1" x="4"/>
-        <item h="1" x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10984,9 +11672,162 @@
   <rowFields count="1">
     <field x="2"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="53">
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i>
+      <x v="39"/>
+    </i>
+    <i>
+      <x v="40"/>
+    </i>
+    <i>
+      <x v="41"/>
+    </i>
+    <i>
+      <x v="42"/>
+    </i>
+    <i>
+      <x v="43"/>
+    </i>
+    <i>
+      <x v="44"/>
+    </i>
+    <i>
+      <x v="45"/>
+    </i>
+    <i>
+      <x v="46"/>
+    </i>
+    <i>
+      <x v="47"/>
+    </i>
+    <i>
+      <x v="48"/>
+    </i>
+    <i>
+      <x v="49"/>
+    </i>
+    <i>
+      <x v="50"/>
+    </i>
+    <i>
+      <x v="51"/>
+    </i>
+    <i>
+      <x v="52"/>
     </i>
     <i t="grand">
       <x/>
@@ -11051,58 +11892,58 @@
     <tabular pivotCacheId="253204613">
       <items count="53">
         <i x="15" s="1"/>
+        <i x="21" s="1"/>
+        <i x="22" s="1"/>
+        <i x="23" s="1"/>
+        <i x="31" s="1"/>
+        <i x="0" s="1"/>
+        <i x="33" s="1"/>
+        <i x="37" s="1"/>
+        <i x="38" s="1"/>
+        <i x="32" s="1"/>
+        <i x="26" s="1"/>
+        <i x="39" s="1"/>
+        <i x="43" s="1"/>
+        <i x="40" s="1"/>
+        <i x="48" s="1"/>
+        <i x="44" s="1"/>
+        <i x="45" s="1"/>
+        <i x="49" s="1"/>
+        <i x="51" s="1"/>
+        <i x="50" s="1"/>
+        <i x="46" s="1"/>
+        <i x="47" s="1"/>
+        <i x="41" s="1"/>
+        <i x="42" s="1"/>
+        <i x="34" s="1"/>
+        <i x="35" s="1"/>
+        <i x="27" s="1"/>
+        <i x="24" s="1"/>
+        <i x="28" s="1"/>
+        <i x="36" s="1"/>
+        <i x="29" s="1"/>
+        <i x="16" s="1"/>
+        <i x="17" s="1"/>
+        <i x="13" s="1"/>
+        <i x="18" s="1"/>
+        <i x="19" s="1"/>
+        <i x="25" s="1"/>
+        <i x="30" s="1"/>
+        <i x="20" s="1"/>
+        <i x="14" s="1"/>
+        <i x="12" s="1"/>
+        <i x="11" s="1"/>
+        <i x="9" s="1"/>
+        <i x="5" s="1"/>
+        <i x="6" s="1"/>
+        <i x="10" s="1"/>
+        <i x="7" s="1"/>
+        <i x="8" s="1"/>
+        <i x="3" s="1"/>
+        <i x="4" s="1"/>
+        <i x="2" s="1"/>
+        <i x="1" s="1"/>
         <i x="52" s="1" nd="1"/>
-        <i x="21" s="1" nd="1"/>
-        <i x="22" s="1" nd="1"/>
-        <i x="23" s="1" nd="1"/>
-        <i x="31" s="1" nd="1"/>
-        <i x="0" s="1" nd="1"/>
-        <i x="33" s="1" nd="1"/>
-        <i x="37" s="1" nd="1"/>
-        <i x="38" s="1" nd="1"/>
-        <i x="32" s="1" nd="1"/>
-        <i x="26" s="1" nd="1"/>
-        <i x="39" s="1" nd="1"/>
-        <i x="43" s="1" nd="1"/>
-        <i x="40" s="1" nd="1"/>
-        <i x="48" s="1" nd="1"/>
-        <i x="44" s="1" nd="1"/>
-        <i x="45" s="1" nd="1"/>
-        <i x="49" s="1" nd="1"/>
-        <i x="51" s="1" nd="1"/>
-        <i x="50" s="1" nd="1"/>
-        <i x="46" s="1" nd="1"/>
-        <i x="47" s="1" nd="1"/>
-        <i x="41" s="1" nd="1"/>
-        <i x="42" s="1" nd="1"/>
-        <i x="34" s="1" nd="1"/>
-        <i x="35" s="1" nd="1"/>
-        <i x="27" s="1" nd="1"/>
-        <i x="24" s="1" nd="1"/>
-        <i x="28" s="1" nd="1"/>
-        <i x="36" s="1" nd="1"/>
-        <i x="29" s="1" nd="1"/>
-        <i x="16" s="1" nd="1"/>
-        <i x="17" s="1" nd="1"/>
-        <i x="13" s="1" nd="1"/>
-        <i x="18" s="1" nd="1"/>
-        <i x="19" s="1" nd="1"/>
-        <i x="25" s="1" nd="1"/>
-        <i x="30" s="1" nd="1"/>
-        <i x="20" s="1" nd="1"/>
-        <i x="14" s="1" nd="1"/>
-        <i x="12" s="1" nd="1"/>
-        <i x="11" s="1" nd="1"/>
-        <i x="9" s="1" nd="1"/>
-        <i x="5" s="1" nd="1"/>
-        <i x="6" s="1" nd="1"/>
-        <i x="10" s="1" nd="1"/>
-        <i x="7" s="1" nd="1"/>
-        <i x="8" s="1" nd="1"/>
-        <i x="3" s="1" nd="1"/>
-        <i x="4" s="1" nd="1"/>
-        <i x="2" s="1" nd="1"/>
-        <i x="1" s="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -11121,10 +11962,10 @@
     <tabular pivotCacheId="253204613">
       <items count="5">
         <i x="1" s="1"/>
-        <i x="0"/>
-        <i x="2"/>
-        <i x="4"/>
-        <i x="3"/>
+        <i x="0" s="1"/>
+        <i x="2" s="1"/>
+        <i x="4" s="1"/>
+        <i x="3" s="1"/>
       </items>
     </tabular>
   </data>
@@ -11142,9 +11983,9 @@
   <data>
     <tabular pivotCacheId="253204613">
       <items count="3">
-        <i x="2"/>
+        <i x="2" s="1"/>
         <i x="0" s="1"/>
-        <i x="1"/>
+        <i x="1" s="1"/>
       </items>
     </tabular>
   </data>
@@ -11162,11 +12003,11 @@
   <data>
     <tabular pivotCacheId="253204613">
       <items count="5">
+        <i x="3"/>
         <i x="1" s="1"/>
         <i x="2"/>
+        <i x="0"/>
         <i x="4"/>
-        <i x="3" nd="1"/>
-        <i x="0" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -11501,7 +12342,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24B18E38-8E63-4DF0-AC28-BAEE67F02126}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
@@ -11526,18 +12367,34 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B4" s="21">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="21">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="21">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="21">
-        <v>1</v>
+      <c r="B7" s="21">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -11575,7 +12432,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="4">
-        <v>7400.0132999999996</v>
+        <v>376999.80689999979</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -11583,7 +12440,7 @@
         <v>50</v>
       </c>
       <c r="B5" s="4">
-        <v>7400.0132999999996</v>
+        <v>376999.80689999979</v>
       </c>
     </row>
   </sheetData>
@@ -11593,7 +12450,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BD95207-E730-45AF-A787-86985A11230D}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
@@ -11621,15 +12478,47 @@
         <v>21</v>
       </c>
       <c r="B4" s="4">
-        <v>7400.0132999999996</v>
+        <v>53399.941500000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4">
+        <v>108799.82340000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="4">
+        <v>101800.29180000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4">
+        <v>73599.781199999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="4">
+        <v>39399.968999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="4">
-        <v>7400.0132999999996</v>
+      <c r="B9" s="4">
+        <v>376999.80690000003</v>
       </c>
     </row>
   </sheetData>
@@ -21203,7 +22092,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE4993A5-250F-4C4F-B9A8-C46E2747D3CE}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
@@ -21247,14 +22136,575 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
-        <v>50</v>
+      <c r="A5" s="20">
+        <v>44874</v>
       </c>
       <c r="B5" s="21">
-        <v>569.66999999999996</v>
+        <v>554.27</v>
       </c>
       <c r="C5" s="21">
         <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="20">
+        <v>44875</v>
+      </c>
+      <c r="B6" s="21">
+        <v>554.27</v>
+      </c>
+      <c r="C6" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="20">
+        <v>44876</v>
+      </c>
+      <c r="B7" s="21">
+        <v>554.27</v>
+      </c>
+      <c r="C7" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="20">
+        <v>44877</v>
+      </c>
+      <c r="B8" s="21">
+        <v>523.48</v>
+      </c>
+      <c r="C8" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="20">
+        <v>44878</v>
+      </c>
+      <c r="B9" s="21">
+        <v>508.08</v>
+      </c>
+      <c r="C9" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="20">
+        <v>44879</v>
+      </c>
+      <c r="B10" s="21">
+        <v>523.48</v>
+      </c>
+      <c r="C10" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="20">
+        <v>44880</v>
+      </c>
+      <c r="B11" s="21">
+        <v>508.08</v>
+      </c>
+      <c r="C11" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="20">
+        <v>44881</v>
+      </c>
+      <c r="B12" s="21">
+        <v>508.08</v>
+      </c>
+      <c r="C12" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="20">
+        <v>44882</v>
+      </c>
+      <c r="B13" s="21">
+        <v>523.48</v>
+      </c>
+      <c r="C13" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="20">
+        <v>44883</v>
+      </c>
+      <c r="B14" s="21">
+        <v>538.88</v>
+      </c>
+      <c r="C14" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="20">
+        <v>44884</v>
+      </c>
+      <c r="B15" s="21">
+        <v>508.08</v>
+      </c>
+      <c r="C15" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="20">
+        <v>44885</v>
+      </c>
+      <c r="B16" s="21">
+        <v>477.29</v>
+      </c>
+      <c r="C16" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="20">
+        <v>44886</v>
+      </c>
+      <c r="B17" s="21">
+        <v>492.69</v>
+      </c>
+      <c r="C17" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="20">
+        <v>44887</v>
+      </c>
+      <c r="B18" s="21">
+        <v>461.89</v>
+      </c>
+      <c r="C18" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="20">
+        <v>44888</v>
+      </c>
+      <c r="B19" s="21">
+        <v>477.29</v>
+      </c>
+      <c r="C19" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="20">
+        <v>44889</v>
+      </c>
+      <c r="B20" s="21">
+        <v>477.29</v>
+      </c>
+      <c r="C20" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="20">
+        <v>44890</v>
+      </c>
+      <c r="B21" s="21">
+        <v>461.89</v>
+      </c>
+      <c r="C21" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="20">
+        <v>44891</v>
+      </c>
+      <c r="B22" s="21">
+        <v>446.5</v>
+      </c>
+      <c r="C22" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="20">
+        <v>44892</v>
+      </c>
+      <c r="B23" s="21">
+        <v>461.89</v>
+      </c>
+      <c r="C23" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="20">
+        <v>44893</v>
+      </c>
+      <c r="B24" s="21">
+        <v>477.29</v>
+      </c>
+      <c r="C24" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="20">
+        <v>44894</v>
+      </c>
+      <c r="B25" s="21">
+        <v>477.29</v>
+      </c>
+      <c r="C25" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="20">
+        <v>44895</v>
+      </c>
+      <c r="B26" s="21">
+        <v>492.69</v>
+      </c>
+      <c r="C26" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="20">
+        <v>44896</v>
+      </c>
+      <c r="B27" s="21">
+        <v>492.69</v>
+      </c>
+      <c r="C27" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="20">
+        <v>44897</v>
+      </c>
+      <c r="B28" s="21">
+        <v>523.48</v>
+      </c>
+      <c r="C28" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="20">
+        <v>44898</v>
+      </c>
+      <c r="B29" s="21">
+        <v>523.48</v>
+      </c>
+      <c r="C29" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="20">
+        <v>44899</v>
+      </c>
+      <c r="B30" s="21">
+        <v>538.88</v>
+      </c>
+      <c r="C30" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="20">
+        <v>44900</v>
+      </c>
+      <c r="B31" s="21">
+        <v>554.27</v>
+      </c>
+      <c r="C31" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="20">
+        <v>44901</v>
+      </c>
+      <c r="B32" s="21">
+        <v>538.88</v>
+      </c>
+      <c r="C32" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="20">
+        <v>44902</v>
+      </c>
+      <c r="B33" s="21">
+        <v>523.48</v>
+      </c>
+      <c r="C33" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="20">
+        <v>44903</v>
+      </c>
+      <c r="B34" s="21">
+        <v>538.88</v>
+      </c>
+      <c r="C34" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="20">
+        <v>44904</v>
+      </c>
+      <c r="B35" s="21">
+        <v>569.66999999999996</v>
+      </c>
+      <c r="C35" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="20">
+        <v>44905</v>
+      </c>
+      <c r="B36" s="21">
+        <v>569.66999999999996</v>
+      </c>
+      <c r="C36" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="20">
+        <v>44906</v>
+      </c>
+      <c r="B37" s="21">
+        <v>585.07000000000005</v>
+      </c>
+      <c r="C37" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="20">
+        <v>44907</v>
+      </c>
+      <c r="B38" s="21">
+        <v>569.66999999999996</v>
+      </c>
+      <c r="C38" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="20">
+        <v>44908</v>
+      </c>
+      <c r="B39" s="21">
+        <v>569.66999999999996</v>
+      </c>
+      <c r="C39" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="20">
+        <v>44909</v>
+      </c>
+      <c r="B40" s="21">
+        <v>554.27</v>
+      </c>
+      <c r="C40" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="20">
+        <v>44910</v>
+      </c>
+      <c r="B41" s="21">
+        <v>538.88</v>
+      </c>
+      <c r="C41" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="20">
+        <v>44911</v>
+      </c>
+      <c r="B42" s="21">
+        <v>569.66999999999996</v>
+      </c>
+      <c r="C42" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="20">
+        <v>44912</v>
+      </c>
+      <c r="B43" s="21">
+        <v>585.07000000000005</v>
+      </c>
+      <c r="C43" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="20">
+        <v>44913</v>
+      </c>
+      <c r="B44" s="21">
+        <v>600.46</v>
+      </c>
+      <c r="C44" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="20">
+        <v>44914</v>
+      </c>
+      <c r="B45" s="21">
+        <v>631.25</v>
+      </c>
+      <c r="C45" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="20">
+        <v>44915</v>
+      </c>
+      <c r="B46" s="21">
+        <v>646.65</v>
+      </c>
+      <c r="C46" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="20">
+        <v>44916</v>
+      </c>
+      <c r="B47" s="21">
+        <v>677.44</v>
+      </c>
+      <c r="C47" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="20">
+        <v>44917</v>
+      </c>
+      <c r="B48" s="21">
+        <v>677.44</v>
+      </c>
+      <c r="C48" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="20">
+        <v>44918</v>
+      </c>
+      <c r="B49" s="21">
+        <v>646.65</v>
+      </c>
+      <c r="C49" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="20">
+        <v>44919</v>
+      </c>
+      <c r="B50" s="21">
+        <v>677.44</v>
+      </c>
+      <c r="C50" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="20">
+        <v>44920</v>
+      </c>
+      <c r="B51" s="21">
+        <v>677.44</v>
+      </c>
+      <c r="C51" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="20">
+        <v>44921</v>
+      </c>
+      <c r="B52" s="21">
+        <v>692.84</v>
+      </c>
+      <c r="C52" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="20">
+        <v>44922</v>
+      </c>
+      <c r="B53" s="21">
+        <v>692.84</v>
+      </c>
+      <c r="C53" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="20">
+        <v>44923</v>
+      </c>
+      <c r="B54" s="21">
+        <v>723.63</v>
+      </c>
+      <c r="C54" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="20">
+        <v>44924</v>
+      </c>
+      <c r="B55" s="21">
+        <v>754.43</v>
+      </c>
+      <c r="C55" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B56" s="21">
+        <v>558.12134615384605</v>
+      </c>
+      <c r="C56" s="21">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>